<commit_message>
Goodness Glamour v2 - Auth, Notifications, Admin Dashboard
</commit_message>
<xml_diff>
--- a/data/contact-messages.xlsx
+++ b/data/contact-messages.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -449,9 +449,29 @@
 </v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>02/05/2026, 11:37 am</v>
+      </c>
+      <c r="B3" t="str">
+        <v>M Sirisha</v>
+      </c>
+      <c r="C3" t="str">
+        <v>9611150532</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Kids Hair Services</v>
+      </c>
+      <c r="E3" t="str">
+        <v>#112 vijnatham south campus, Adichunchanagiri ayurvedic medical college,nagarur</v>
+      </c>
+      <c r="F3" t="str">
+        <v xml:space="preserve">want hair spa and conditioning </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>